<commit_message>
Phase 3: people and contracts, map, executive brief and reporting calendar
- Staff extracted from report workbooks (Purchase Orders + GL sheets), classified
  Local / SxB-HQ, merged per person; coverage, renewals, contract confirmation
  with manual overrides; People tab on project pages
- Offline bubble map with country cards and sector mix
- Printable executive brief and contractual reporting calendar
- Fix uppercase headings rendering with Turkish dotted I (page language)
- Month arithmetic clamps to month end; tests for staff, deadlines and flows

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PAqPek3YRKEsiyNM1yxxoY
</commit_message>
<xml_diff>
--- a/next/tests/fixtures/report-q3.xlsx
+++ b/next/tests/fixtures/report-q3.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchase Orders" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,185 +436,305 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>1.1 Local staff (Ankara)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>Language Rights Programme</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Approved budget</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Staff</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1860000</v>
+      </c>
+      <c r="D5" t="n">
+        <v>900000</v>
+      </c>
+      <c r="E5" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>372000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>180000</v>
+      </c>
+      <c r="E6" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Equipment and services</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2170000</v>
+      </c>
+      <c r="D7" t="n">
+        <v>700000</v>
+      </c>
+      <c r="E7" t="n">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Local office</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>310000</v>
+      </c>
+      <c r="D8" t="n">
+        <v>120000</v>
+      </c>
+      <c r="E8" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Other costs</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>930000</v>
+      </c>
+      <c r="D9" t="n">
+        <v>300000</v>
+      </c>
+      <c r="E9" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Indirect costs</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>558000</v>
+      </c>
+      <c r="D10" t="n">
+        <v>200000</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>6200000</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="E11" t="n">
+        <v>175000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Purchase orders</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Reporting line</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Description PO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PO number</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Spent in EUR</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Spent and committed in EUR</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>No.</t>
+          <t>1.1.1.4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Testova, Ayla - Project officer from 01/01/2026 to 31/10/2026 100%</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Approved budget</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Actual</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Committed</t>
-        </is>
+          <t>4599001</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E3" t="n">
+        <v>9000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.2.1.2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Staff</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1860000</v>
+          <t>Example, Max - Project manager from 01/03/2026 to 28/02/2027 50%</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>4599002</t>
+        </is>
       </c>
       <c r="D4" t="n">
-        <v>900000</v>
+        <v>4000</v>
       </c>
       <c r="E4" t="n">
-        <v>50000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.1.1.7</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Travel</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>372000</v>
-      </c>
-      <c r="D5" t="n">
-        <v>180000</v>
-      </c>
-      <c r="E5" t="n">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Equipment and services</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>2170000</v>
-      </c>
-      <c r="D6" t="n">
-        <v>700000</v>
-      </c>
-      <c r="E6" t="n">
-        <v>90000</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Local office</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>310000</v>
-      </c>
-      <c r="D7" t="n">
-        <v>120000</v>
-      </c>
-      <c r="E7" t="n">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Other costs</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>930000</v>
-      </c>
-      <c r="D8" t="n">
-        <v>300000</v>
-      </c>
-      <c r="E8" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Indirect costs</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>558000</v>
-      </c>
-      <c r="D9" t="n">
-        <v>200000</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>6200000</v>
-      </c>
-      <c r="D10" t="n">
-        <v>2400000</v>
-      </c>
-      <c r="E10" t="n">
-        <v>175000</v>
-      </c>
+          <t>Unreadable row</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>4599003</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>